<commit_message>
updation of test data
</commit_message>
<xml_diff>
--- a/POS_Lanes_TestData.xlsx
+++ b/POS_Lanes_TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BanuchandhiranM\Git\POS_Lanes_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7E1617B-D4E0-4058-98CE-AF9631F3FA17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4DA005B-A158-42D0-A4BC-136D5A8E777A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10" yWindow="10" windowWidth="19190" windowHeight="11270" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="237" uniqueCount="180">
   <si>
     <t>fileName</t>
   </si>
@@ -202,9 +202,6 @@
   </si>
   <si>
     <t>VfQueryUpdate.exe</t>
-  </si>
-  <si>
-    <t>PASS</t>
   </si>
   <si>
     <t xml:space="preserve">Diebold Nixdorf | Diebold Nixdorf Universal TouchDriver | 2.2.14 </t>
@@ -1378,7 +1375,7 @@
         <v>37</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
   </sheetData>
@@ -1647,10 +1644,10 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="23" t="s">
+        <v>130</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>131</v>
-      </c>
-      <c r="B1" s="23" t="s">
-        <v>132</v>
       </c>
       <c r="C1" s="23" t="s">
         <v>3</v>
@@ -1658,15 +1655,15 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B2" t="s">
         <v>133</v>
-      </c>
-      <c r="B2" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B3" s="24">
         <v>45973.791666666664</v>
@@ -1674,74 +1671,74 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" t="s">
         <v>136</v>
-      </c>
-      <c r="B4" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B6" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B11" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>
@@ -1763,16 +1760,16 @@
   <sheetData>
     <row r="1" spans="1:5" s="23" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="C1" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="23" t="s">
         <v>128</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>129</v>
       </c>
       <c r="E1" s="23" t="s">
         <v>3</v>
@@ -1780,43 +1777,43 @@
     </row>
     <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="21" t="s">
         <v>60</v>
-      </c>
-      <c r="B2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
+        <v>123</v>
+      </c>
+      <c r="C3" s="21" t="s">
         <v>62</v>
-      </c>
-      <c r="B3" t="s">
-        <v>124</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" s="21" t="s">
         <v>64</v>
-      </c>
-      <c r="B4" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C5" s="21">
         <v>3.22</v>
@@ -1824,186 +1821,186 @@
     </row>
     <row r="6" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="19" t="s">
+        <v>166</v>
+      </c>
+      <c r="C6" s="21" t="s">
         <v>66</v>
-      </c>
-      <c r="B6" s="19" t="s">
-        <v>167</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B7" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="C7" s="21" t="s">
         <v>68</v>
-      </c>
-      <c r="B7" s="19" t="s">
-        <v>166</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="B8" s="19" t="s">
+        <v>164</v>
+      </c>
+      <c r="C8" s="21" t="s">
         <v>70</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>165</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="C9" s="21" t="s">
         <v>72</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="19" t="s">
+        <v>73</v>
+      </c>
+      <c r="B10" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="C10" s="21" t="s">
         <v>74</v>
-      </c>
-      <c r="B10" s="19" t="s">
-        <v>163</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="B11" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="C11" s="21" t="s">
         <v>76</v>
-      </c>
-      <c r="B11" s="19" t="s">
-        <v>162</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="19" t="s">
+        <v>77</v>
+      </c>
+      <c r="B12" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="C12" s="21" t="s">
         <v>78</v>
-      </c>
-      <c r="B12" s="19" t="s">
-        <v>161</v>
-      </c>
-      <c r="C12" s="21" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="B13" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13" s="21" t="s">
         <v>80</v>
-      </c>
-      <c r="B13" s="19" t="s">
-        <v>160</v>
-      </c>
-      <c r="C13" s="21" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="19" t="s">
+        <v>81</v>
+      </c>
+      <c r="B14" s="19" t="s">
+        <v>158</v>
+      </c>
+      <c r="C14" s="21" t="s">
         <v>82</v>
-      </c>
-      <c r="B14" s="19" t="s">
-        <v>159</v>
-      </c>
-      <c r="C14" s="21" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="19" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C15" s="21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="19" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="C16" s="21" t="s">
         <v>85</v>
-      </c>
-      <c r="B16" s="19" t="s">
-        <v>157</v>
-      </c>
-      <c r="C16" s="21" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="C17" s="21" t="s">
         <v>87</v>
-      </c>
-      <c r="B17" s="19" t="s">
-        <v>156</v>
-      </c>
-      <c r="C17" s="21" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="19" t="s">
+        <v>88</v>
+      </c>
+      <c r="B18" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="C18" s="21" t="s">
         <v>89</v>
-      </c>
-      <c r="B18" s="19" t="s">
-        <v>155</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="C19" s="21" t="s">
         <v>91</v>
-      </c>
-      <c r="B19" s="19" t="s">
-        <v>154</v>
-      </c>
-      <c r="C19" s="21" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="19" t="s">
+        <v>92</v>
+      </c>
+      <c r="B20" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="C20" s="21" t="s">
         <v>93</v>
-      </c>
-      <c r="B20" s="19" t="s">
-        <v>153</v>
-      </c>
-      <c r="C20" s="21" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="19" t="s">
+        <v>94</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>151</v>
+      </c>
+      <c r="C21" s="21" t="s">
         <v>95</v>
-      </c>
-      <c r="B21" s="19" t="s">
-        <v>152</v>
-      </c>
-      <c r="C21" s="21" t="s">
-        <v>96</v>
       </c>
     </row>
     <row r="22" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C22" s="21">
         <v>2023</v>
@@ -2011,153 +2008,153 @@
     </row>
     <row r="23" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>168</v>
+      </c>
+      <c r="C23" s="21" t="s">
         <v>98</v>
-      </c>
-      <c r="B23" s="19" t="s">
-        <v>169</v>
-      </c>
-      <c r="C23" s="21" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="19" t="s">
+        <v>99</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="C24" s="21" t="s">
         <v>100</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>172</v>
-      </c>
-      <c r="C24" s="21" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="B26" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="C26" s="21" t="s">
         <v>103</v>
-      </c>
-      <c r="B26" s="19" t="s">
-        <v>171</v>
-      </c>
-      <c r="C26" s="21" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="19" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="28" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="B28" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="C28" s="21" t="s">
         <v>106</v>
-      </c>
-      <c r="B28" s="19" t="s">
-        <v>174</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="29" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="19" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="B30" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="C30" s="21" t="s">
         <v>109</v>
-      </c>
-      <c r="B30" s="19" t="s">
-        <v>176</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="B31" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="C31" s="21" t="s">
         <v>111</v>
-      </c>
-      <c r="B31" s="19" t="s">
-        <v>177</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="28.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="19" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C32" s="21" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="C33" s="21" t="s">
         <v>114</v>
-      </c>
-      <c r="B33" s="19" t="s">
-        <v>179</v>
-      </c>
-      <c r="C33" s="21" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="19" t="s">
+        <v>115</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>148</v>
+      </c>
+      <c r="C34" s="21" t="s">
         <v>116</v>
-      </c>
-      <c r="B34" s="19" t="s">
-        <v>149</v>
-      </c>
-      <c r="C34" s="21" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="B35" t="s">
+        <v>147</v>
+      </c>
+      <c r="C35" s="21" t="s">
         <v>118</v>
-      </c>
-      <c r="B35" t="s">
-        <v>148</v>
-      </c>
-      <c r="C35" s="21" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="19" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B36" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C36" s="21">
         <v>2</v>
@@ -2165,13 +2162,13 @@
     </row>
     <row r="37" spans="1:3" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37" s="21" t="s">
         <v>121</v>
-      </c>
-      <c r="B37" t="s">
-        <v>146</v>
-      </c>
-      <c r="C37" s="21" t="s">
-        <v>122</v>
       </c>
     </row>
   </sheetData>
@@ -2196,16 +2193,16 @@
   <sheetData>
     <row r="1" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="18" t="s">
+        <v>125</v>
+      </c>
+      <c r="B1" s="23" t="s">
         <v>126</v>
       </c>
-      <c r="B1" s="23" t="s">
+      <c r="C1" s="20" t="s">
         <v>127</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="23" t="s">
         <v>128</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>129</v>
       </c>
       <c r="E1" s="23" t="s">
         <v>3</v>
@@ -2215,38 +2212,35 @@
     </row>
     <row r="2" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="B2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C2" s="21" t="s">
         <v>60</v>
-      </c>
-      <c r="B2" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" s="21" t="s">
-        <v>61</v>
-      </c>
-      <c r="E2" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="19" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" t="s">
+        <v>129</v>
+      </c>
+      <c r="C3" s="21" t="s">
         <v>62</v>
-      </c>
-      <c r="B3" t="s">
-        <v>130</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B4" t="s">
+        <v>124</v>
+      </c>
+      <c r="C4" s="21" t="s">
         <v>64</v>
-      </c>
-      <c r="B4" t="s">
-        <v>125</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>